<commit_message>
docs(qa): migrate historical test cases [SPARK-177][SPARK-181][SPARK-197][SPARK-314]
</commit_message>
<xml_diff>
--- a/docs/04-testing/test-cases/SmartParking_Facility_Master_TestCases.xlsx
+++ b/docs/04-testing/test-cases/SmartParking_Facility_Master_TestCases.xlsx
@@ -2,10 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Re40185392d1b4c2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="2" r:id="Re53d4181650247cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case List" sheetId="3" r:id="Ra86d54f2857241d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration Queue" sheetId="4" r:id="R5bf1365cd19b4b5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R134eeb0646c24548"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="2" r:id="R682373262682493f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case List" sheetId="3" r:id="R31f22332a43c4f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration Queue" sheetId="4" r:id="R5e22201031b24855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR9_Facility_UI" sheetId="5" r:id="Ra2fe9416c05c41a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ownership_Audit" sheetId="6" r:id="R14405039f4454a92"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
+    <x:numFmt numFmtId="201" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -42,8 +45,37 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17354A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF2B4552"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF0C4D68"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF15384A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -70,6 +102,31 @@
         <x:fgColor rgb="FFEAF3EA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF102A3B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD7E8EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F2F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF183C52"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDECF2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -78,7 +135,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -139,10 +196,68 @@
     <x:xf numFmtId="200" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="2">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFDE8E8"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE6F5EB"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
@@ -413,7 +528,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>1.0 DRAFT</x:v>
+        <x:v>1.1 REVIEW</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -459,6 +574,26 @@
       </x:c>
       <x:c r="G12" s="26" t="str">
         <x:v>Mentor TestTeam_UAT.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="B13" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>Migrate PR9 Facility UI</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>2 UI PASS, API origin to confirm</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>PR9_QA_Traceability_Final.xlsx</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -597,10 +732,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>No executed cases recorded</x:v>
+        <x:v>PR9_Facility_UI</x:v>
       </x:c>
       <x:c r="D11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E11" t="n">
         <x:v>0</x:v>
@@ -612,44 +747,46 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I11" s="32" t="n">
-        <x:v>0</x:v>
+        <x:f>IFERROR(D11/H11,0)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="C12" s="29" t="str">
+      <x:c r="B12" s="56"/>
+      <x:c r="C12" s="56" t="str">
         <x:v>Sub total</x:v>
       </x:c>
-      <x:c r="D12" s="29" t="n">
+      <x:c r="D12" s="56" t="n">
         <x:f>SUM(D11:D11)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E12" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E12" s="56" t="n">
         <x:f>SUM(E11:E11)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F12" s="29" t="n">
+      <x:c r="F12" s="56" t="n">
         <x:f>SUM(F11:F11)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G12" s="29" t="n">
+      <x:c r="G12" s="56" t="n">
         <x:f>SUM(G11:G11)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H12" s="29" t="n">
+      <x:c r="H12" s="56" t="n">
         <x:f>SUM(H11:H11)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I12" s="33" t="n">
-        <x:f>IF(H12=0,0,D12/H12)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J12" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I12" s="57" t="n">
+        <x:f>IFERROR(D12/H12,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J12" s="56" t="n">
         <x:f>SUM(J11:J11)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -659,8 +796,8 @@
         <x:v>QA execution coverage</x:v>
       </x:c>
       <x:c r="C22" s="32" t="n">
-        <x:f>IF(H12=0,0,(D12+E12)/H12)</x:f>
-        <x:v>0</x:v>
+        <x:f>IFERROR((D12+E12)/H12,0)</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -668,7 +805,7 @@
         <x:v>Status / sign-off</x:v>
       </x:c>
       <x:c r="C23" t="str">
-        <x:v>No executed cases imported; pending historical evidence</x:v>
+        <x:v>2 PR9 UI checks reported PASS on 05e2976d; ownership provisional. No Facility backend API pass claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -684,7 +821,7 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>Mentor TestTeam_UAT.xlsx; PR14 QA logs (2026-10-27)</x:v>
+        <x:v>PR9_QA_Traceability_Final.xlsx; PR9_QA_Final_Report.docx; source screenshots in Word appendix.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="35" customHeight="1">
@@ -793,15 +930,21 @@
         <x:v>Pre-Condition</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="B9"/>
-      <x:c r="C9"/>
-      <x:c r="D9"/>
-      <x:c r="E9" t="str">
-        <x:v>No cases loaded yet; see Migration Queue for historical backlog.</x:v>
-      </x:c>
-      <x:c r="F9" t="str">
-        <x:v>Evidence pending</x:v>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="B9" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="26" t="str">
+        <x:v>PR9_Facility_UI</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="str">
+        <x:v>PR9_Facility_UI</x:v>
+      </x:c>
+      <x:c r="E9" s="26" t="str">
+        <x:v>Owner site list and site-filter dashboard UI</x:v>
+      </x:c>
+      <x:c r="F9" s="26" t="str">
+        <x:v>Authenticated Owner with assigned QA site</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -856,16 +999,425 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="B6"/>
+      <x:c r="B6" t="str">
+        <x:v>PR9 / Facility UI</x:v>
+      </x:c>
       <x:c r="C6" t="str">
-        <x:v>No verified historical cases imported</x:v>
-      </x:c>
-      <x:c r="D6"/>
+        <x:v>Owner Site list + Dashboard site filter (2 checks)</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>2 PASS limited to UI display at SHA 05e2976d; no network trace available in historical ZIP.</x:v>
+      </x:c>
       <x:c r="E6" t="str">
-        <x:v>Wait for original task/evidence and root-service attribution</x:v>
+        <x:v>Ownership provisional: confirm originating frontend API call, avoid duplicate entries in User master.</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>2 FACILITY UI CASES / OWNERSHIP REVIEW</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="B1:F1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="48" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="25" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="25" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="48" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="35" customHeight="1">
+      <x:c r="B1" s="39" t="str">
+        <x:v>SMART PARKING  |  PR9_Facility_UI</x:v>
+      </x:c>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
+      <x:c r="F1" s="39"/>
+      <x:c r="G1" s="39"/>
+      <x:c r="H1" s="39"/>
+      <x:c r="I1" s="39"/>
+      <x:c r="J1" s="39"/>
+      <x:c r="K1" s="39"/>
+      <x:c r="L1" s="39"/>
+      <x:c r="M1" s="39"/>
+      <x:c r="N1" s="39"/>
+      <x:c r="O1" s="39"/>
+      <x:c r="P1" s="39"/>
+      <x:c r="Q1" s="39"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="B2" s="41" t="str">
+        <x:v>Module Code</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>PR9_Facility_UI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="B3" s="41" t="str">
+        <x:v>Test requirement</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>PR #9 · QA candidate SPARK-182 (provisional; confirm service root/API call chain)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="B4" s="41" t="str">
+        <x:v>Reference Document</x:v>
+      </x:c>
+      <x:c r="C4" s="44" t="str">
+        <x:v>Two Site/Dashboard UI-only checks from PR9; provisionally classified to Facility as likely initiator. No backend API proof.</x:v>
+      </x:c>
+      <x:c r="D4" s="44"/>
+      <x:c r="E4" s="44"/>
+      <x:c r="F4" s="44"/>
+      <x:c r="G4" s="44"/>
+      <x:c r="H4" s="44"/>
+      <x:c r="I4" s="44"/>
+      <x:c r="J4" s="44"/>
+      <x:c r="K4" s="44"/>
+      <x:c r="L4" s="44"/>
+      <x:c r="M4" s="44"/>
+      <x:c r="N4" s="44"/>
+      <x:c r="O4" s="44"/>
+      <x:c r="P4" s="44"/>
+      <x:c r="Q4" s="44"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="B5" s="49" t="str">
+        <x:v>% Passed of tests</x:v>
+      </x:c>
+      <x:c r="C5" s="49" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D5" s="49" t="str">
+        <x:v>Fail</x:v>
+      </x:c>
+      <x:c r="E5" s="49" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="F5" s="49" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="G5" s="49" t="str">
+        <x:v>Number of test cases</x:v>
+      </x:c>
+      <x:c r="H5" s="49" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="B6" s="32" t="n">
+        <x:f>IFERROR(C6/G6,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="B8" s="44" t="str">
+        <x:v>Nguồn: tài liệu gốc trong Historical ZIP. Tổng hợp theo nhiều commit; không suy diễn kết quả ở HEAD mới.</x:v>
+      </x:c>
+      <x:c r="C8" s="44"/>
+      <x:c r="D8" s="44"/>
+      <x:c r="E8" s="44"/>
+      <x:c r="F8" s="44"/>
+      <x:c r="G8" s="44"/>
+      <x:c r="H8" s="44"/>
+      <x:c r="I8" s="44"/>
+      <x:c r="J8" s="44"/>
+      <x:c r="K8" s="44"/>
+      <x:c r="L8" s="44"/>
+      <x:c r="M8" s="44"/>
+      <x:c r="N8" s="44"/>
+      <x:c r="O8" s="44"/>
+      <x:c r="P8" s="44"/>
+      <x:c r="Q8" s="44"/>
+    </x:row>
+    <x:row r="9" ht="35" customHeight="1">
+      <x:c r="B9" s="49" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="C9" s="49" t="str">
+        <x:v>Test Case Description</x:v>
+      </x:c>
+      <x:c r="D9" s="49" t="str">
+        <x:v>Test Case Procedure</x:v>
+      </x:c>
+      <x:c r="E9" s="49" t="str">
+        <x:v>Expected Results</x:v>
+      </x:c>
+      <x:c r="F9" s="49" t="str">
+        <x:v>Inter-test case Dependence</x:v>
+      </x:c>
+      <x:c r="G9" s="49" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="H9" s="49" t="str">
+        <x:v>Test date</x:v>
+      </x:c>
+      <x:c r="I9" s="49" t="str">
+        <x:v>Tester</x:v>
+      </x:c>
+      <x:c r="J9" s="49" t="str">
+        <x:v>Number of tests</x:v>
+      </x:c>
+      <x:c r="K9" s="49" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L9" s="49" t="str">
+        <x:v>% Passed</x:v>
+      </x:c>
+      <x:c r="M9" s="49" t="str">
+        <x:v>Note / Actual</x:v>
+      </x:c>
+      <x:c r="N9" s="49" t="str">
+        <x:v>Testing Jira</x:v>
+      </x:c>
+      <x:c r="O9" s="49" t="str">
+        <x:v>Baseline commit</x:v>
+      </x:c>
+      <x:c r="P9" s="49" t="str">
+        <x:v>Evidence / source</x:v>
+      </x:c>
+      <x:c r="Q9" s="49" t="str">
+        <x:v>Scenario type</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="57" customHeight="1">
+      <x:c r="B10" s="52" t="str">
+        <x:v>[PR9-R22-07]</x:v>
+      </x:c>
+      <x:c r="C10" s="26" t="str">
+        <x:v>Owner Site list</x:v>
+      </x:c>
+      <x:c r="D10" s="26" t="str">
+        <x:v>Site &amp; Staff Management</x:v>
+      </x:c>
+      <x:c r="E10" s="26" t="str">
+        <x:v>Facility displayed + ACTIVE</x:v>
+      </x:c>
+      <x:c r="F10" s="26" t="str">
+        <x:v>Owner logged in</x:v>
+      </x:c>
+      <x:c r="G10" s="26" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H10" s="26" t="str">
+        <x:v>2026-10-22</x:v>
+      </x:c>
+      <x:c r="I10" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J10" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K10" s="26" t="n">
+        <x:f>IF(G10="Pass",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L10" s="51" t="n">
+        <x:f>IFERROR(K10/J10,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M10" s="26" t="str">
+        <x:v>PR9 QA SMTP Test Lot; ACTIVE; 0 physical slots
+PASS is limited to displayed Site/Facility UI. Facility service ownership provisional until API call-chain is checked. Physical layout chưa tạo</x:v>
+      </x:c>
+      <x:c r="N10" s="26" t="str">
+        <x:v>SPARK-182 candidate (provisional; verify service root and scope)</x:v>
+      </x:c>
+      <x:c r="O10" s="26" t="str">
+        <x:v>05e2976d (short SHA, source-reported)</x:v>
+      </x:c>
+      <x:c r="P10" s="26" t="str">
+        <x:v>EV-OWNER-OLD · PR9_QA_Traceability_Final.xlsx TEST_CASES; Word screenshot index</x:v>
+      </x:c>
+      <x:c r="Q10" s="26" t="str">
+        <x:v>Facility UI (provisional service ownership; verify actual API request chain)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="57" customHeight="1">
+      <x:c r="B11" s="52" t="str">
+        <x:v>[PR9-R22-08]</x:v>
+      </x:c>
+      <x:c r="C11" s="26" t="str">
+        <x:v>Owner Dashboard</x:v>
+      </x:c>
+      <x:c r="D11" s="26" t="str">
+        <x:v>Select PR9 QA SMTP Test Lot at Site filter</x:v>
+      </x:c>
+      <x:c r="E11" s="26" t="str">
+        <x:v>Dashboard filters correct facility</x:v>
+      </x:c>
+      <x:c r="F11" s="26" t="str">
+        <x:v>Owner logged in; site present</x:v>
+      </x:c>
+      <x:c r="G11" s="26" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H11" s="26" t="str">
+        <x:v>2026-10-22</x:v>
+      </x:c>
+      <x:c r="I11" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J11" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K11" s="26" t="n">
+        <x:f>IF(G11="Pass",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L11" s="51" t="n">
+        <x:f>IFERROR(K11/J11,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M11" s="26" t="str">
+        <x:v>Filtered site view; Capacity 0
+PASS is limited to displayed Site/Facility UI. Facility service ownership provisional until API call-chain is checked. Capacity driven by saved physical layout</x:v>
+      </x:c>
+      <x:c r="N11" s="26" t="str">
+        <x:v>SPARK-182 candidate (provisional; verify service root and scope)</x:v>
+      </x:c>
+      <x:c r="O11" s="26" t="str">
+        <x:v>05e2976d (short SHA, source-reported)</x:v>
+      </x:c>
+      <x:c r="P11" s="26" t="str">
+        <x:v>EV-OWNER-OLD · PR9_QA_Traceability_Final.xlsx TEST_CASES; Word screenshot index</x:v>
+      </x:c>
+      <x:c r="Q11" s="26" t="str">
+        <x:v>Facility UI (provisional service ownership; verify actual API request chain)</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="B1:Q1"/>
+    <x:mergeCell ref="C4:Q4"/>
+    <x:mergeCell ref="B8:Q8"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="G10:G11">
+    <x:cfRule type="expression" dxfId="0" priority="1">
+      <x:formula>G10="Fail"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="1" priority="2">
+      <x:formula>G10="Pass"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G10:G11">
+      <x:formula1>"Pass,Fail,Untested,Blocked,N/A"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="B1" s="39" t="str">
+        <x:v>OWNERSHIP AUDIT</x:v>
+      </x:c>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
+      <x:c r="F1" s="39"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="B3" s="49" t="str">
+        <x:v>Case ID</x:v>
+      </x:c>
+      <x:c r="C3" s="49" t="str">
+        <x:v>Provisional root</x:v>
+      </x:c>
+      <x:c r="D3" s="49" t="str">
+        <x:v>Observed UI scope</x:v>
+      </x:c>
+      <x:c r="E3" s="49" t="str">
+        <x:v>Why provisional</x:v>
+      </x:c>
+      <x:c r="F3" s="49" t="str">
+        <x:v>Required check</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="53" customHeight="1">
+      <x:c r="B4" s="26" t="str">
+        <x:v>PR9-R22-07</x:v>
+      </x:c>
+      <x:c r="C4" s="26" t="str">
+        <x:v>Facility (candidate)</x:v>
+      </x:c>
+      <x:c r="D4" s="26" t="str">
+        <x:v>Owner Site &amp; Staff Management shows ACTIVE QA site</x:v>
+      </x:c>
+      <x:c r="E4" s="26" t="str">
+        <x:v>No DevTools request trace in source ZIP</x:v>
+      </x:c>
+      <x:c r="F4" s="26" t="str">
+        <x:v>SPARK-182 is candidate testing Jira, pending verification of original API initiator.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="53" customHeight="1">
+      <x:c r="B5" s="26" t="str">
+        <x:v>PR9-R22-08</x:v>
+      </x:c>
+      <x:c r="C5" s="26" t="str">
+        <x:v>Facility (candidate)</x:v>
+      </x:c>
+      <x:c r="D5" s="26" t="str">
+        <x:v>Owner Dashboard site filter displays QA site</x:v>
+      </x:c>
+      <x:c r="E5" s="26" t="str">
+        <x:v>Could involve User/Facility read-model aggregation</x:v>
+      </x:c>
+      <x:c r="F5" s="26" t="str">
+        <x:v>SPARK-182 candidate, do not claim Facility backend API tested.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>